<commit_message>
Add GitHub-backed feedback storage
</commit_message>
<xml_diff>
--- a/SNAP_Bivariate _Classification_Dataset.xlsx
+++ b/SNAP_Bivariate _Classification_Dataset.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nowsh\Downloads\Research\Fall 2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nowsh\Downloads\Research\Fall 2025\food_insecurity_dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87E77604-C311-41EC-9F1D-A2F6F66D6B5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8E68379-A32C-44C0-A34B-344868896114}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{85984DDD-8E03-4E71-BB7D-ACE5956AC118}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10658" uniqueCount="1580">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10658" uniqueCount="1581">
   <si>
     <t>fips</t>
   </si>
@@ -4786,6 +4786,9 @@
   </si>
   <si>
     <t>Moderate Need</t>
+  </si>
+  <si>
+    <t>Average Increase in Visit</t>
   </si>
 </sst>
 </file>
@@ -27194,7 +27197,7 @@
         <v>1564</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>7</v>
+        <v>1580</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>8</v>

</xml_diff>